<commit_message>
fix(word/table): stop flagging consumed 'data' key as unsupported
The inline 'data' shorthand (--prop data=A,B;1,2) is consumed up-front by
TryGetValue("data") to build the grid, but the later tblPr switch loop had no
skip/case for it, so its default branch pushed 'data' into LastAddUnsupportedProps
— a spurious unsupported_property WARNING on a key that worked. Add 'data' to the
same skip-list that already excludes rows/cols/colwidths (all consumed elsewhere).
Genuine typos still warn.

Also closes the word tables example: demonstrate the 'data' shorthand (Table 7),
taking table@docx coverage to 19/19. Fixed a pre-existing breakage in tables.sh
where the PPTX section used the rejected '/presentation/slides' parent instead of
'/', so tables.pptx never rebuilt. Regenerated docx/xlsx/pptx — all open in real
Office (officeshot) and validate clean. Table test suite green (1887).
</commit_message>
<xml_diff>
--- a/examples/word/tables.xlsx
+++ b/examples/word/tables.xlsx
@@ -3,8 +3,8 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="Performance" sheetId="2" r:id="R461334ad036f4383"/>
-    <x:sheet name="Summary" sheetId="3" r:id="Re51b8710c20049ed"/>
+    <x:sheet name="Performance" sheetId="2" r:id="R714f79221d3447af"/>
+    <x:sheet name="Summary" sheetId="3" r:id="R9fa1b3db10c244e9"/>
   </x:sheets>
   <x:calcPr fullCalcOnLoad="1"/>
 </x:workbook>

</xml_diff>